<commit_message>
Updated to new convention
</commit_message>
<xml_diff>
--- a/Raw_to_JSON.xlsx
+++ b/Raw_to_JSON.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11013"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Adrian Metlenko\Dropbox (Bench)\BENCH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adrian/Documents/Personal/Pesnik.db/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38493BAF-4E41-4CC9-9D6B-C649DC85132A}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C5C4D21-7E1D-DC49-92F0-AEE524C182AE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10536" yWindow="1488" windowWidth="17280" windowHeight="9024" xr2:uid="{3B3296F3-CFAF-43B5-A5FB-1B474682DE3E}"/>
+    <workbookView xWindow="25600" yWindow="460" windowWidth="25600" windowHeight="28340" xr2:uid="{3B3296F3-CFAF-43B5-A5FB-1B474682DE3E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
   <si>
     <t xml:space="preserve">    "Россия — любимая наша страна.",</t>
   </si>
@@ -103,67 +103,70 @@
     <t>xxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxxx</t>
   </si>
   <si>
-    <t>Слышу старой песни мотив,</t>
-  </si>
-  <si>
-    <t>что сама напевала не раз</t>
-  </si>
-  <si>
-    <t>И глаза закрываю на миг, забыв,</t>
-  </si>
-  <si>
-    <t>что я городская сейчас</t>
-  </si>
-  <si>
-    <t>Эта песня синий простор</t>
-  </si>
-  <si>
-    <t>край родимый напомнила мне</t>
-  </si>
-  <si>
-    <t>И девчонку ту, что с недавних пор</t>
-  </si>
-  <si>
-    <t>часто вижу я во сне</t>
-  </si>
-  <si>
-    <t>Хуто-хуторянка,</t>
-  </si>
-  <si>
-    <t>девчоночка смуглянка</t>
-  </si>
-  <si>
-    <t>Мне бы хоть разок</t>
-  </si>
-  <si>
-    <t>всего лишь на чуток</t>
-  </si>
-  <si>
-    <t>Мою весну на хуторок</t>
-  </si>
-  <si>
-    <t>Медом дышит лунная ночь</t>
-  </si>
-  <si>
-    <t>редкий свет из окошек домов</t>
-  </si>
-  <si>
-    <t>И как хочется снова сорваться прочь</t>
-  </si>
-  <si>
-    <t>в сиреневый рай садов</t>
-  </si>
-  <si>
-    <t>Чтобы кругом опять голова</t>
-  </si>
-  <si>
-    <t>и слова как хмельное вино</t>
-  </si>
-  <si>
-    <t>Чтобы ночь была - не расти трава,</t>
-  </si>
-  <si>
-    <t>любишь-губишь все равно</t>
+    <t>На недельку до второго</t>
+  </si>
+  <si>
+    <t>Я уеду в Комарово</t>
+  </si>
+  <si>
+    <t>Поглядеть отвыкшим глазом</t>
+  </si>
+  <si>
+    <t>На балтийскую волну.</t>
+  </si>
+  <si>
+    <t>И на море буду разом</t>
+  </si>
+  <si>
+    <t>Кораблём и водолазом,</t>
+  </si>
+  <si>
+    <t>Сам себя найду в пучине,</t>
+  </si>
+  <si>
+    <t>Если часом затону.</t>
+  </si>
+  <si>
+    <t>Я уеду в Комарово,</t>
+  </si>
+  <si>
+    <t>Сам себя найду в пучине</t>
+  </si>
+  <si>
+    <t>Где качается на дюнах</t>
+  </si>
+  <si>
+    <t>Шереметьевский баркас.</t>
+  </si>
+  <si>
+    <t>И у вас в карельских скалах</t>
+  </si>
+  <si>
+    <t>На общественных началах,</t>
+  </si>
+  <si>
+    <t>Если только захотите,</t>
+  </si>
+  <si>
+    <t>Будет личный водолаз.</t>
+  </si>
+  <si>
+    <t>На воскресной электричке</t>
+  </si>
+  <si>
+    <t>К вам на краешек земли.</t>
+  </si>
+  <si>
+    <t>Водолазы ищут клады,</t>
+  </si>
+  <si>
+    <t>Только кладов мне не надо,</t>
+  </si>
+  <si>
+    <t>Я за то, чтоб в синем море</t>
+  </si>
+  <si>
+    <t>Не тонули корабли.</t>
   </si>
 </sst>
 </file>
@@ -206,27 +209,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="62">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="60">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1138,16 +1121,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{712BC2BD-F9A5-42FF-85D8-C454A7B6B32A}">
   <dimension ref="A1:E61"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="80" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.77734375" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" customWidth="1"/>
-    <col min="4" max="4" width="13.77734375" customWidth="1"/>
-    <col min="5" max="5" width="43.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.5" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="43.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1164,10 +1147,10 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="str">
-        <f>CONCATENATE( "    {",CHAR(34),"break",CHAR(34),":",LOWER(B2),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C2),",",CHAR(34),"repeat",CHAR(34),":",LOWER(D2),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E2,CHAR(34),"},")</f>
-        <v xml:space="preserve">    {"break":true,"chorus":false,"repeat":false,"lyric_line":"Слышу старой песни мотив,"},</v>
+        <f>CONCATENATE( "    {",CHAR(34),"space",CHAR(34),":",LOWER(B2),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C2),",",CHAR(34),"x_repeat",CHAR(34),":",LOWER(D2),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E2,CHAR(34),"},")</f>
+        <v xml:space="preserve">    {"space":true,"chorus":false,"x_repeat":false,"lyric_line":"На недельку до второго"},</v>
       </c>
       <c r="B2" t="b">
         <v>1</v>
@@ -1182,10 +1165,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="str">
-        <f t="shared" ref="A3:A17" si="0">CONCATENATE( "    {",CHAR(34),"break",CHAR(34),":",LOWER(B3),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C3),",",CHAR(34),"repeat",CHAR(34),":",LOWER(D3),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E3,CHAR(34),"},")</f>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"что сама напевала не раз"},</v>
+        <f t="shared" ref="A3:A61" si="0">CONCATENATE( "    {",CHAR(34),"space",CHAR(34),":",LOWER(B3),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C3),",",CHAR(34),"x_repeat",CHAR(34),":",LOWER(D3),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E3,CHAR(34),"},")</f>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Я уеду в Комарово"},</v>
       </c>
       <c r="B3" t="b">
         <v>0</v>
@@ -1200,10 +1183,10 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"И глаза закрываю на миг, забыв,"},</v>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Поглядеть отвыкшим глазом"},</v>
       </c>
       <c r="B4" t="b">
         <v>0</v>
@@ -1218,10 +1201,10 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"что я городская сейчас"},</v>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"На балтийскую волну."},</v>
       </c>
       <c r="B5" t="b">
         <v>0</v>
@@ -1236,10 +1219,10 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":true,"chorus":false,"repeat":false,"lyric_line":"Эта песня синий простор"},</v>
+        <v xml:space="preserve">    {"space":true,"chorus":false,"x_repeat":false,"lyric_line":"И на море буду разом"},</v>
       </c>
       <c r="B6" t="b">
         <v>1</v>
@@ -1254,10 +1237,10 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"край родимый напомнила мне"},</v>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Кораблём и водолазом,"},</v>
       </c>
       <c r="B7" t="b">
         <v>0</v>
@@ -1272,10 +1255,10 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"И девчонку ту, что с недавних пор"},</v>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Сам себя найду в пучине,"},</v>
       </c>
       <c r="B8" t="b">
         <v>0</v>
@@ -1290,10 +1273,10 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"часто вижу я во сне"},</v>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Если часом затону."},</v>
       </c>
       <c r="B9" t="b">
         <v>0</v>
@@ -1308,10 +1291,10 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":true,"chorus":true,"repeat":true,"lyric_line":"Хуто-хуторянка,"},</v>
+        <v xml:space="preserve">    {"space":true,"chorus":true,"x_repeat":false,"lyric_line":"На недельку до второго"},</v>
       </c>
       <c r="B10" t="b">
         <v>1</v>
@@ -1320,250 +1303,250 @@
         <v>1</v>
       </c>
       <c r="D10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":false,"lyric_line":"Я уеду в Комарово,"},</v>
+      </c>
+      <c r="B11" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" t="b">
+        <v>0</v>
+      </c>
+      <c r="E11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":"девчоночка смуглянка"},</v>
-      </c>
-      <c r="B11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C11" t="b">
-        <v>1</v>
-      </c>
-      <c r="D11" t="b">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":false,"lyric_line":"Сам себя найду в пучине"},</v>
+      </c>
+      <c r="B12" t="b">
+        <v>0</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":"Мне бы хоть разок"},</v>
-      </c>
-      <c r="B12" t="b">
-        <v>0</v>
-      </c>
-      <c r="C12" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" t="b">
-        <v>1</v>
-      </c>
-      <c r="E12" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":false,"lyric_line":"Если часом затону."},</v>
+      </c>
+      <c r="B13" t="b">
+        <v>0</v>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" t="b">
+        <v>0</v>
+      </c>
+      <c r="E13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":true,"chorus":false,"x_repeat":false,"lyric_line":"На недельку до второго"},</v>
+      </c>
+      <c r="B14" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Я уеду в Комарово,"},</v>
+      </c>
+      <c r="B15" t="b">
+        <v>0</v>
+      </c>
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Где качается на дюнах"},</v>
+      </c>
+      <c r="B16" t="b">
+        <v>0</v>
+      </c>
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
+      <c r="E16" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":"всего лишь на чуток"},</v>
-      </c>
-      <c r="B13" t="b">
-        <v>0</v>
-      </c>
-      <c r="C13" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" t="b">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Шереметьевский баркас."},</v>
+      </c>
+      <c r="B17" t="b">
+        <v>0</v>
+      </c>
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":"Мою весну на хуторок"},</v>
-      </c>
-      <c r="B14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C14" t="b">
-        <v>1</v>
-      </c>
-      <c r="D14" t="b">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":true,"chorus":false,"x_repeat":false,"lyric_line":"И у вас в карельских скалах"},</v>
+      </c>
+      <c r="B18" t="b">
+        <v>1</v>
+      </c>
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":true,"chorus":false,"repeat":false,"lyric_line":"Медом дышит лунная ночь"},</v>
-      </c>
-      <c r="B15" t="b">
-        <v>1</v>
-      </c>
-      <c r="C15" t="b">
-        <v>0</v>
-      </c>
-      <c r="D15" t="b">
-        <v>0</v>
-      </c>
-      <c r="E15" t="s">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"На общественных началах,"},</v>
+      </c>
+      <c r="B19" t="b">
+        <v>0</v>
+      </c>
+      <c r="C19" t="b">
+        <v>0</v>
+      </c>
+      <c r="D19" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"редкий свет из окошек домов"},</v>
-      </c>
-      <c r="B16" t="b">
-        <v>0</v>
-      </c>
-      <c r="C16" t="b">
-        <v>0</v>
-      </c>
-      <c r="D16" t="b">
-        <v>0</v>
-      </c>
-      <c r="E16" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Если только захотите,"},</v>
+      </c>
+      <c r="B20" t="b">
+        <v>0</v>
+      </c>
+      <c r="C20" t="b">
+        <v>0</v>
+      </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"И как хочется снова сорваться прочь"},</v>
-      </c>
-      <c r="B17" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17" t="b">
-        <v>0</v>
-      </c>
-      <c r="D17" t="b">
-        <v>0</v>
-      </c>
-      <c r="E17" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Будет личный водолаз."},</v>
+      </c>
+      <c r="B21" t="b">
+        <v>0</v>
+      </c>
+      <c r="C21" t="b">
+        <v>0</v>
+      </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="str">
-        <f t="shared" ref="A3:A29" si="1">CONCATENATE( "    {",CHAR(34),"break",CHAR(34),":",LOWER(B18),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C18),",",CHAR(34),"repeat",CHAR(34),":",LOWER(D18),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E18,CHAR(34),"},")</f>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"в сиреневый рай садов"},</v>
-      </c>
-      <c r="B18" t="b">
-        <v>0</v>
-      </c>
-      <c r="C18" t="b">
-        <v>0</v>
-      </c>
-      <c r="D18" t="b">
-        <v>0</v>
-      </c>
-      <c r="E18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":true,"chorus":false,"repeat":false,"lyric_line":"Чтобы кругом опять голова"},</v>
-      </c>
-      <c r="B19" t="b">
-        <v>1</v>
-      </c>
-      <c r="C19" t="b">
-        <v>0</v>
-      </c>
-      <c r="D19" t="b">
-        <v>0</v>
-      </c>
-      <c r="E19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"и слова как хмельное вино"},</v>
-      </c>
-      <c r="B20" t="b">
-        <v>0</v>
-      </c>
-      <c r="C20" t="b">
-        <v>0</v>
-      </c>
-      <c r="D20" t="b">
-        <v>0</v>
-      </c>
-      <c r="E20" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"Чтобы ночь была - не расти трава,"},</v>
-      </c>
-      <c r="B21" t="b">
-        <v>0</v>
-      </c>
-      <c r="C21" t="b">
-        <v>0</v>
-      </c>
-      <c r="D21" t="b">
-        <v>0</v>
-      </c>
-      <c r="E21" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":"любишь-губишь все равно"},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":true,"chorus":true,"x_repeat":false,"lyric_line":"На недельку до второго"},</v>
       </c>
       <c r="B22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" t="b">
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":true,"chorus":true,"repeat":true,"lyric_line":"Хуто-хуторянка,"},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":false,"lyric_line":"Я уеду в Комарово,"},</v>
       </c>
       <c r="B23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C23" t="b">
         <v>1</v>
       </c>
       <c r="D23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":"девчоночка смуглянка"},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":false,"lyric_line":"И у вас в карельских скалах"},</v>
       </c>
       <c r="B24" t="b">
         <v>0</v>
@@ -1572,16 +1555,16 @@
         <v>1</v>
       </c>
       <c r="D24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E24" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":"Мне бы хоть разок"},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":false,"lyric_line":"Будет личный водолаз."},</v>
       </c>
       <c r="B25" t="b">
         <v>0</v>
@@ -1590,97 +1573,106 @@
         <v>1</v>
       </c>
       <c r="D25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":"всего лишь на чуток"},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":true,"chorus":false,"x_repeat":false,"lyric_line":"На недельку до второго"},</v>
       </c>
       <c r="B26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":"Мою весну на хуторок"},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Я уеду в Комарово"},</v>
       </c>
       <c r="B27" t="b">
         <v>0</v>
       </c>
       <c r="C27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"На воскресной электричке"},</v>
       </c>
       <c r="B28" t="b">
         <v>0</v>
       </c>
       <c r="C28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E28" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"К вам на краешек земли."},</v>
       </c>
       <c r="B29" t="b">
         <v>0</v>
       </c>
       <c r="C29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E29" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="str">
-        <f t="shared" ref="A3:A33" si="2">CONCATENATE( "    {",CHAR(34),"break",CHAR(34),":",LOWER(B30),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C30),",",CHAR(34),"repeat",CHAR(34),":",LOWER(D30),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E30,CHAR(34),"},")</f>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":true,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":true,"chorus":false,"x_repeat":false,"lyric_line":"Водолазы ищут клады,"},</v>
       </c>
       <c r="B30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" t="b">
         <v>0</v>
       </c>
       <c r="D30" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":true,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Только кладов мне не надо,"},</v>
       </c>
       <c r="B31" t="b">
         <v>0</v>
@@ -1689,13 +1681,16 @@
         <v>0</v>
       </c>
       <c r="D31" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":true,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Я за то, чтоб в синем море"},</v>
       </c>
       <c r="B32" t="b">
         <v>0</v>
@@ -1704,13 +1699,16 @@
         <v>0</v>
       </c>
       <c r="D32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="str">
-        <f t="shared" si="2"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":true,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":"Не тонули корабли."},</v>
       </c>
       <c r="B33" t="b">
         <v>0</v>
@@ -1719,76 +1717,91 @@
         <v>0</v>
       </c>
       <c r="D33" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="str">
-        <f t="shared" ref="A34:A45" si="3">CONCATENATE( "    {",CHAR(34),"break",CHAR(34),":",LOWER(B34),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C34),",",CHAR(34),"repeat",CHAR(34),":",LOWER(D34),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E34,CHAR(34),"},")</f>
-        <v xml:space="preserve">    {"break":true,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":true,"chorus":true,"x_repeat":true,"lyric_line":"На недельку до второго"},</v>
       </c>
       <c r="B34" t="b">
         <v>1</v>
       </c>
       <c r="C34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E34" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":true,"lyric_line":"Я уеду в Комарово,"},</v>
       </c>
       <c r="B35" t="b">
         <v>0</v>
       </c>
       <c r="C35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E35" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":true,"lyric_line":"Я за то, чтоб в синем море"},</v>
       </c>
       <c r="B36" t="b">
         <v>0</v>
       </c>
       <c r="C36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E36" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":true,"x_repeat":true,"lyric_line":"Не тонули корабли."},</v>
       </c>
       <c r="B37" t="b">
         <v>0</v>
       </c>
       <c r="C37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D37" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+      <c r="E37" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":true,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C38" t="b">
         <v>0</v>
@@ -1797,10 +1810,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B39" t="b">
         <v>0</v>
@@ -1812,10 +1825,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B40" t="b">
         <v>0</v>
@@ -1827,10 +1840,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B41" t="b">
         <v>0</v>
@@ -1842,193 +1855,193 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":true,"chorus":true,"repeat":true,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D42" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B43" t="b">
         <v>0</v>
       </c>
       <c r="C43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B44" t="b">
         <v>0</v>
       </c>
       <c r="C44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="str">
-        <f t="shared" si="3"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":true,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B45" t="b">
         <v>0</v>
       </c>
       <c r="C45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="str">
-        <f t="shared" ref="A46:A49" si="4">CONCATENATE( "    {",CHAR(34),"break",CHAR(34),":",LOWER(B46),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C46),",",CHAR(34),"repeat",CHAR(34),":",LOWER(D46),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E46,CHAR(34),"},")</f>
-        <v xml:space="preserve">    {"break":true,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D46" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B47" t="b">
         <v>0</v>
       </c>
       <c r="C47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D47" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B48" t="b">
         <v>0</v>
       </c>
       <c r="C48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="str">
-        <f t="shared" si="4"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B49" t="b">
         <v>0</v>
       </c>
       <c r="C49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D49" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="str">
-        <f t="shared" ref="A50:A61" si="5">CONCATENATE( "    {",CHAR(34),"break",CHAR(34),":",LOWER(B50),",",CHAR(34),"chorus",CHAR(34),":",LOWER(C50),",",CHAR(34),"repeat",CHAR(34),":",LOWER(D50),",",CHAR(34),"lyric_line",CHAR(34),":",CHAR(34),E50,CHAR(34),"},")</f>
-        <v xml:space="preserve">    {"break":true,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D50" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B51" t="b">
         <v>0</v>
       </c>
       <c r="C51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D51" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B52" t="b">
         <v>0</v>
       </c>
       <c r="C52" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D52" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":true,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B53" t="b">
         <v>0</v>
       </c>
       <c r="C53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D53" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":true,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C54" t="b">
         <v>0</v>
@@ -2037,10 +2050,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B55" t="b">
         <v>0</v>
@@ -2052,10 +2065,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B56" t="b">
         <v>0</v>
@@ -2067,10 +2080,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B57" t="b">
         <v>0</v>
@@ -2082,13 +2095,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":true,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B58" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C58" t="b">
         <v>0</v>
@@ -2097,10 +2110,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B59" t="b">
         <v>0</v>
@@ -2112,10 +2125,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B60" t="b">
         <v>0</v>
@@ -2127,10 +2140,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="str">
-        <f t="shared" si="5"/>
-        <v xml:space="preserve">    {"break":false,"chorus":false,"repeat":false,"lyric_line":""},</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">    {"space":false,"chorus":false,"x_repeat":false,"lyric_line":""},</v>
       </c>
       <c r="B61" t="b">
         <v>0</v>
@@ -2143,135 +2156,23 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C62:D1048576 D50:D61 C1:D5 B2:B5">
-    <cfRule type="cellIs" dxfId="61" priority="941" operator="equal">
+  <conditionalFormatting sqref="C62:D1048576 D61 B2:B13 C1:D13 B38:D60">
+    <cfRule type="cellIs" dxfId="59" priority="965" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="942" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="966" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B58:C61">
-    <cfRule type="cellIs" dxfId="59" priority="503" operator="equal">
+  <conditionalFormatting sqref="B61:C61">
+    <cfRule type="cellIs" dxfId="57" priority="527" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="504" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="528" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B54:C57">
-    <cfRule type="cellIs" dxfId="57" priority="505" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="506" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B50:C53">
-    <cfRule type="cellIs" dxfId="55" priority="409" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="410" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B46:D49">
-    <cfRule type="cellIs" dxfId="53" priority="269" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="270" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B34:B37 C34:D45">
-    <cfRule type="cellIs" dxfId="51" priority="51" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="52" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B38:B41">
-    <cfRule type="cellIs" dxfId="49" priority="49" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="50" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B42:B45 D42:D45">
-    <cfRule type="cellIs" dxfId="47" priority="47" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="48" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B34:B37 D34:D41">
-    <cfRule type="cellIs" dxfId="45" priority="45" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="46" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B38:B41">
-    <cfRule type="cellIs" dxfId="43" priority="43" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="44" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B42:B45">
-    <cfRule type="cellIs" dxfId="41" priority="41" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="42" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B30:D33">
-    <cfRule type="cellIs" dxfId="35" priority="35" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="36" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B28:D29">
-    <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="16" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:D9">
-    <cfRule type="cellIs" dxfId="13" priority="13" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="14" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B10:D14">
-    <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="12" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B15:D18">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B19:D22">
+  <conditionalFormatting sqref="B14:D25">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2279,7 +2180,7 @@
       <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23:D27">
+  <conditionalFormatting sqref="B26:D37">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2295,94 +2196,94 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCA2DBD8-617B-41B3-90F3-3CA278E48793}">
   <dimension ref="B1:B18"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>16</v>
       </c>

</xml_diff>